<commit_message>
Add configurable team assets and improve settings UX
</commit_message>
<xml_diff>
--- a/data/partecipanti_example.xlsx
+++ b/data/partecipanti_example.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partecipanti" sheetId="1" r:id="R0b2f10fa566c402b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partecipanti" sheetId="1" r:id="Rc7327243fafa4bc5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -374,7 +374,7 @@
         <x:v>Rossi</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>ROSSI</x:v>
+        <x:v>FENICI</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -388,7 +388,7 @@
         <x:v>Rossi</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>BLU</x:v>
+        <x:v>DRAGHI</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -402,7 +402,7 @@
         <x:v>Bianchi</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>BLU</x:v>
+        <x:v>DRAGHI</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -416,7 +416,7 @@
         <x:v>Verdi</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>GIALLI</x:v>
+        <x:v>TITANI</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -430,7 +430,7 @@
         <x:v>Bianchi</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>BLU</x:v>
+        <x:v>DRAGHI</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -444,7 +444,7 @@
         <x:v>Romano</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>VERDI</x:v>
+        <x:v>GRIFONI</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -458,7 +458,7 @@
         <x:v>Pellegrini</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>ROSSI</x:v>
+        <x:v>FENICI</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -472,7 +472,7 @@
         <x:v>Pellicciotta</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>BLU</x:v>
+        <x:v>DRAGHI</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -486,7 +486,7 @@
         <x:v>De Luca</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>GIALLI</x:v>
+        <x:v>TITANI</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -500,7 +500,7 @@
         <x:v>De Angelis</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>VERDI</x:v>
+        <x:v>GRIFONI</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -514,13 +514,13 @@
         <x:v>Romani</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>ROSSI</x:v>
+        <x:v>FENICI</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4b705f3a89e40d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13643070406d466b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>